<commit_message>
update code and traits data
</commit_message>
<xml_diff>
--- a/traits_data.xlsx
+++ b/traits_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10118"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joaobiosmac/Desktop/Trabalhos &amp; Repositórios/Artigos em Andamento/Cap 3A e 3B/Cap 3A/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joaobiosmac/Desktop/Trabalhos &amp; Repositórios/Artigos em Andamento/Cap 3A e 3B/Cap 4/Cap4_repo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2949883-8FD0-CF4E-821A-17D8F51B3138}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C904420B-98FA-1243-9896-3EE6D620A075}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1660" yWindow="1160" windowWidth="26020" windowHeight="14300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="128">
   <si>
     <t>Relative_eye_position</t>
   </si>
@@ -76,9 +76,6 @@
     <t>Synbranchus marmoratus</t>
   </si>
   <si>
-    <t>ARR</t>
-  </si>
-  <si>
     <t>CTMax</t>
   </si>
   <si>
@@ -106,102 +103,51 @@
     <t>33.5333333333333</t>
   </si>
   <si>
-    <t>1.88034188034188</t>
-  </si>
-  <si>
     <t>37.4754901960784</t>
   </si>
   <si>
-    <t>0.820130475302889</t>
-  </si>
-  <si>
     <t>37.575</t>
   </si>
   <si>
-    <t>0.388035569927243</t>
-  </si>
-  <si>
     <t>35.3068181818182</t>
   </si>
   <si>
-    <t>1.52215799614644</t>
-  </si>
-  <si>
     <t>32.625</t>
   </si>
   <si>
-    <t>2.17582417582418</t>
-  </si>
-  <si>
     <t>35.16</t>
   </si>
   <si>
-    <t>0.747185261003071</t>
-  </si>
-  <si>
     <t>34.4375</t>
   </si>
   <si>
-    <t>0.909090909090908</t>
-  </si>
-  <si>
-    <t>2.46268656716418</t>
-  </si>
-  <si>
     <t>34.5818181818182</t>
   </si>
   <si>
-    <t>2.48447204968944</t>
-  </si>
-  <si>
     <t>39.05</t>
   </si>
   <si>
-    <t>0.857142857142858</t>
-  </si>
-  <si>
     <t>34.05</t>
   </si>
   <si>
-    <t>1.09</t>
-  </si>
-  <si>
     <t>35.0333333333333</t>
   </si>
   <si>
-    <t>0.609375</t>
-  </si>
-  <si>
     <t>32.95</t>
   </si>
   <si>
-    <t>3.88</t>
-  </si>
-  <si>
     <t>33.825</t>
   </si>
   <si>
-    <t>0.793201133144475</t>
-  </si>
-  <si>
     <t>35.2095238095238</t>
   </si>
   <si>
-    <t>2.7735368956743</t>
-  </si>
-  <si>
     <t>36.275</t>
   </si>
   <si>
-    <t>0.793650793650794</t>
-  </si>
-  <si>
     <t>37.0666666666667</t>
   </si>
   <si>
-    <t>0.788912579957355</t>
-  </si>
-  <si>
     <t>35.21</t>
   </si>
   <si>
@@ -455,9 +401,6 @@
   </si>
   <si>
     <t>0.18</t>
-  </si>
-  <si>
-    <t>0.28627451</t>
   </si>
   <si>
     <t>Atlantirivulus peruibensis</t>
@@ -543,7 +486,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -555,9 +498,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -877,7 +817,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26.6640625" customWidth="1"/>
@@ -888,615 +828,557 @@
     <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="8" width="20.5" customWidth="1"/>
     <col min="9" max="9" width="18.5" customWidth="1"/>
-    <col min="10" max="10" width="25.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>21</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>22</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="4" t="s">
-        <v>24</v>
-      </c>
       <c r="I1" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="J1" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>65</v>
+        <v>47</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>69</v>
+        <v>51</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
       <c r="H2" s="3">
         <v>1</v>
       </c>
-      <c r="I2" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="I2" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+      <c r="A4" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="I3" s="8" t="s">
+      <c r="G4" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="I4" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="J3" s="5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="10" t="s">
-        <v>146</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="I4" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="I5" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="D6" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="E6" s="3" t="s">
-        <v>91</v>
-      </c>
       <c r="F6" s="3" t="s">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="I6" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>43</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>69</v>
+        <v>51</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>96</v>
+        <v>78</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>97</v>
+        <v>79</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="I7" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>99</v>
+        <v>81</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="H8" s="3">
         <v>1</v>
       </c>
-      <c r="I8" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="J8" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="I8" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>107</v>
-      </c>
       <c r="G9" s="3" t="s">
-        <v>108</v>
+        <v>90</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="I9" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="J9" s="5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>58</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>97</v>
+        <v>79</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>110</v>
+        <v>92</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="I10" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="J10" s="5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>93</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>112</v>
+        <v>94</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>113</v>
+        <v>95</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>114</v>
+        <v>96</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="I11" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="J11" s="5" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>117</v>
+        <v>99</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>118</v>
+        <v>100</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="I12" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+      <c r="A13" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="D13" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="J12" s="5" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A13" s="9" t="s">
-        <v>139</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>62</v>
-      </c>
       <c r="E13" s="3" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>121</v>
+        <v>103</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="I13" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="J13" s="5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>104</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>123</v>
+        <v>105</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>124</v>
+        <v>106</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>97</v>
+        <v>79</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>125</v>
+        <v>107</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>126</v>
+        <v>108</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>127</v>
+        <v>109</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="I14" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="J14" s="5" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>140</v>
+        <v>122</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>141</v>
+        <v>123</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>69</v>
+        <v>51</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>127</v>
+        <v>109</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="I15" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="J15" s="5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>46</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>128</v>
+        <v>110</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>129</v>
+        <v>111</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>130</v>
+        <v>112</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>131</v>
+        <v>113</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="I16" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="J16" s="5" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>114</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>133</v>
+        <v>115</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>134</v>
+        <v>116</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>135</v>
+        <v>117</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="I17" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="J17" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>137</v>
+        <v>119</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>132</v>
+        <v>114</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>135</v>
+        <v>117</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="I18" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="J18" s="5" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>120</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>17</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>64</v>
+        <v>46</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>142</v>
+        <v>124</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>132</v>
+        <v>114</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>143</v>
+        <v>125</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="I19" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="J19" s="5" t="s">
-        <v>59</v>
+        <v>126</v>
+      </c>
+      <c r="I19" s="7" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>